<commit_message>
Ladezeit beim Einlesen der Fahrerkarte
</commit_message>
<xml_diff>
--- a/Dokumentation.xlsx
+++ b/Dokumentation.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20401"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54C7948D-C147-4174-925D-2BD46F6A681E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21E9BA63-8698-4BBC-948A-A38E6B6A3155}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variablen" sheetId="2" r:id="rId1"/>
@@ -1757,6 +1757,45 @@
     <t>Ziel-Page nach Ablauf der Wartezeit</t>
   </si>
   <si>
+    <t>nuntius_printer_visLoadingInfo</t>
+  </si>
+  <si>
+    <t>Informationstext auf dem Ladebildschrim</t>
+  </si>
+  <si>
+    <t>nuntius_printer_ui_loadingInfo</t>
+  </si>
+  <si>
+    <t>Lade- und Fehlermeldungsinfotext</t>
+  </si>
+  <si>
+    <t>nuntius_printer_updateWaitTimer</t>
+  </si>
+  <si>
+    <t>Aktualisiert den Wartezeit-Timer für die Simulation von Ladezeiten</t>
+  </si>
+  <si>
+    <t>nuntius_printer_startWaitTime</t>
+  </si>
+  <si>
+    <t>nuntius_printer_goToPageAfterWaitTime</t>
+  </si>
+  <si>
+    <t>Öffnet die "Bitte Warten"-Seite für die Ladezeit-Simulation</t>
+  </si>
+  <si>
+    <t>Wartezeit in Sekunden</t>
+  </si>
+  <si>
+    <t>Wait-Reason für die Ladezeit</t>
+  </si>
+  <si>
+    <t>Zielseite nach Ablauf der Wartezeit</t>
+  </si>
+  <si>
+    <t>Startet die Wartezeit mit dem gegebenen Wartegrund</t>
+  </si>
+  <si>
     <t>Enum-Wert für den Grund der Wartezeit, die gestartet wurde.
 -1 = undefiniert
 0 = Fahrerkarte einlesen
@@ -1766,46 +1805,8 @@
 4 = Ziel prüfen
 5 = Warten auf Ticketdruck
 6 = Pause aktivieren
-7 = Abmelden</t>
-  </si>
-  <si>
-    <t>nuntius_printer_visLoadingInfo</t>
-  </si>
-  <si>
-    <t>Informationstext auf dem Ladebildschrim</t>
-  </si>
-  <si>
-    <t>nuntius_printer_ui_loadingInfo</t>
-  </si>
-  <si>
-    <t>Lade- und Fehlermeldungsinfotext</t>
-  </si>
-  <si>
-    <t>nuntius_printer_updateWaitTimer</t>
-  </si>
-  <si>
-    <t>Aktualisiert den Wartezeit-Timer für die Simulation von Ladezeiten</t>
-  </si>
-  <si>
-    <t>nuntius_printer_startWaitTime</t>
-  </si>
-  <si>
-    <t>nuntius_printer_goToPageAfterWaitTime</t>
-  </si>
-  <si>
-    <t>Öffnet die "Bitte Warten"-Seite für die Ladezeit-Simulation</t>
-  </si>
-  <si>
-    <t>Wartezeit in Sekunden</t>
-  </si>
-  <si>
-    <t>Wait-Reason für die Ladezeit</t>
-  </si>
-  <si>
-    <t>Zielseite nach Ablauf der Wartezeit</t>
-  </si>
-  <si>
-    <t>Startet die Wartezeit mit dem gegebenen Wartegrund</t>
+7 = Abmelden
+10 = Fahrerkarte nach der Pause einlesen</t>
   </si>
 </sst>
 </file>
@@ -2476,12 +2477,12 @@
         <v>350</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="165" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" ht="181.5" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>550</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>556</v>
+        <v>569</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
@@ -2760,10 +2761,10 @@
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="B86" s="3" t="s">
         <v>557</v>
-      </c>
-      <c r="B86" s="3" t="s">
-        <v>558</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.3">
@@ -3160,10 +3161,10 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>559</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>560</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
@@ -3910,10 +3911,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>560</v>
+      </c>
+      <c r="B32" t="s">
         <v>561</v>
-      </c>
-      <c r="B32" t="s">
-        <v>562</v>
       </c>
       <c r="C32" t="s">
         <v>251</v>
@@ -4342,30 +4343,30 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
+        <v>563</v>
+      </c>
+      <c r="B81" t="s">
         <v>564</v>
       </c>
-      <c r="B81" t="s">
+      <c r="D81" t="s">
         <v>565</v>
       </c>
-      <c r="D81" t="s">
-        <v>566</v>
-      </c>
       <c r="E81" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B82" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="D82" t="s">
+        <v>565</v>
+      </c>
+      <c r="E82" t="s">
         <v>566</v>
-      </c>
-      <c r="E82" t="s">
-        <v>567</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
@@ -4462,7 +4463,7 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B96" s="13"/>
       <c r="D96" s="13"/>

</xml_diff>